<commit_message>
Se realizo la correccion de los archivos SCPM-05 y SCPM-07.
</commit_message>
<xml_diff>
--- a/backend/outputs/50693032/50693032_EVENTO_SCPM-07.xlsx
+++ b/backend/outputs/50693032/50693032_EVENTO_SCPM-07.xlsx
@@ -2129,7 +2129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q57"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.5703125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -2762,26 +2762,7 @@
           <t>264067</t>
         </is>
       </c>
-      <c r="N30" s="131" t="inlineStr">
-        <is>
-          <t>589850</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>554435</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>558738</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>390918</t>
-        </is>
-      </c>
+      <c r="N30" s="131" t="n"/>
     </row>
     <row r="31" ht="102" customHeight="1">
       <c r="A31" s="172" t="n"/>
@@ -2817,26 +2798,7 @@
           <t>Patricio Baltazar Angel</t>
         </is>
       </c>
-      <c r="N31" s="131" t="inlineStr">
-        <is>
-          <t>Perez Reyes Bryan</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Ramirez Garduño Jesus Alberto</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>Salgado Garcia Selene Berenice</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>Sampayo Davila Luis Alberto</t>
-        </is>
-      </c>
+      <c r="N31" s="131" t="n"/>
     </row>
     <row r="32" ht="16.5" customHeight="1">
       <c r="A32" s="69" t="inlineStr">

</xml_diff>